<commit_message>
Adding code and excel files
</commit_message>
<xml_diff>
--- a/Excel_Files/sum_states_2.xlsx
+++ b/Excel_Files/sum_states_2.xlsx
@@ -1,51 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uao365-my.sharepoint.com/personal/a1947793_adelaide_edu_au/Documents/JugglingProject_Bukhari_SyedUzairShah_a1947793/Excel_Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="122" documentId="8_{904477D2-7475-DB46-AB97-1B1480DED8CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE067EDD-123F-6042-8061-56170940B74E}"/>
+  <xr:revisionPtr revIDLastSave="132" documentId="8_{904477D2-7475-DB46-AB97-1B1480DED8CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CBCB46C-5F6D-0F4D-8912-91B8807CEF32}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" activeTab="6" xr2:uid="{2BF0295C-3557-5E4A-9758-0F8E5E26ADEC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="3" state="hidden" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="2" state="hidden" r:id="rId3"/>
     <sheet name="exp 4" sheetId="4" state="hidden" r:id="rId4"/>
-    <sheet name="Sheet5" sheetId="6" r:id="rId5"/>
-    <sheet name="Sheet7" sheetId="8" r:id="rId6"/>
-    <sheet name="Sheet6" sheetId="7" r:id="rId7"/>
+    <sheet name="Sheet7" sheetId="8" state="hidden" r:id="rId5"/>
+    <sheet name="raw values" sheetId="6" r:id="rId6"/>
+    <sheet name="summarized values" sheetId="7" r:id="rId7"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v2.0" hidden="1">Sheet6!$D$1</definedName>
-    <definedName name="_xlchart.v2.1" hidden="1">Sheet6!$D$2:$D$5</definedName>
-    <definedName name="_xlchart.v2.10" hidden="1">Sheet6!$D$1:$H$1</definedName>
-    <definedName name="_xlchart.v2.11" hidden="1">Sheet6!$D$2:$H$2</definedName>
-    <definedName name="_xlchart.v2.12" hidden="1">Sheet6!$D$3:$H$3</definedName>
-    <definedName name="_xlchart.v2.13" hidden="1">Sheet6!$D$4:$H$4</definedName>
-    <definedName name="_xlchart.v2.14" hidden="1">Sheet6!$D$5:$H$5</definedName>
-    <definedName name="_xlchart.v2.2" hidden="1">Sheet6!$E$1</definedName>
-    <definedName name="_xlchart.v2.3" hidden="1">Sheet6!$E$2:$E$5</definedName>
-    <definedName name="_xlchart.v2.4" hidden="1">Sheet6!$F$1</definedName>
-    <definedName name="_xlchart.v2.5" hidden="1">Sheet6!$F$2:$F$5</definedName>
-    <definedName name="_xlchart.v2.6" hidden="1">Sheet6!$G$1</definedName>
-    <definedName name="_xlchart.v2.7" hidden="1">Sheet6!$G$2:$G$5</definedName>
-    <definedName name="_xlchart.v2.8" hidden="1">Sheet6!$H$1</definedName>
-    <definedName name="_xlchart.v2.9" hidden="1">Sheet6!$H$2:$H$5</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="11" r:id="rId8"/>
-    <pivotCache cacheId="16" r:id="rId9"/>
-    <pivotCache cacheId="20" r:id="rId10"/>
-    <pivotCache cacheId="24" r:id="rId11"/>
-    <pivotCache cacheId="28" r:id="rId12"/>
-    <pivotCache cacheId="33" r:id="rId13"/>
+    <pivotCache cacheId="16" r:id="rId8"/>
+    <pivotCache cacheId="17" r:id="rId9"/>
+    <pivotCache cacheId="18" r:id="rId10"/>
+    <pivotCache cacheId="19" r:id="rId11"/>
+    <pivotCache cacheId="20" r:id="rId12"/>
+    <pivotCache cacheId="21" r:id="rId13"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -3062,7 +3045,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="170" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -3118,7 +3101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3133,12 +3116,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -3243,7 +3225,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet6!$E$1</c:f>
+              <c:f>'summarized values'!$E$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3264,7 +3246,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet6!$D$2:$D$5</c:f>
+              <c:f>'summarized values'!$D$2:$D$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -3285,7 +3267,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet6!$E$2:$E$5</c:f>
+              <c:f>'summarized values'!$E$2:$E$5</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="4"/>
@@ -3315,7 +3297,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet6!$F$1</c:f>
+              <c:f>'summarized values'!$F$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3336,7 +3318,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet6!$D$2:$D$5</c:f>
+              <c:f>'summarized values'!$D$2:$D$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -3357,7 +3339,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet6!$F$2:$F$5</c:f>
+              <c:f>'summarized values'!$F$2:$F$5</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="4"/>
@@ -3387,7 +3369,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet6!$G$1</c:f>
+              <c:f>'summarized values'!$G$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3408,7 +3390,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet6!$D$2:$D$5</c:f>
+              <c:f>'summarized values'!$D$2:$D$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -3429,7 +3411,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet6!$G$2:$G$5</c:f>
+              <c:f>'summarized values'!$G$2:$G$5</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="4"/>
@@ -3459,7 +3441,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet6!$H$1</c:f>
+              <c:f>'summarized values'!$H$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3480,7 +3462,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet6!$D$2:$D$5</c:f>
+              <c:f>'summarized values'!$D$2:$D$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -3501,7 +3483,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet6!$H$2:$H$5</c:f>
+              <c:f>'summarized values'!$H$2:$H$5</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="4"/>
@@ -4269,16 +4251,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>690880</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>106680</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>365760</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>121920</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>167640</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>904240</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>147320</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4304,6 +4286,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4335,7 +4321,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="SYED UZAIR SHAH BUKHARI - 15020" refreshedDate="46235.712437037037" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="20" xr:uid="{1852F765-E73D-FE40-B217-24C6A55D4B6A}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="C2:D22" sheet="Sheet5"/>
+    <worksheetSource ref="C2:D22" sheet="raw values"/>
   </cacheSource>
   <cacheFields count="2">
     <cacheField name="Prob" numFmtId="0">
@@ -4361,7 +4347,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="SYED UZAIR SHAH BUKHARI - 15020" refreshedDate="46235.71262395833" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="20" xr:uid="{C4F35A6B-B681-1342-96F0-590E7B30AFAF}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="G2:H22" sheet="Sheet5"/>
+    <worksheetSource ref="G2:H22" sheet="raw values"/>
   </cacheSource>
   <cacheFields count="2">
     <cacheField name="Prob" numFmtId="0">
@@ -4387,7 +4373,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="SYED UZAIR SHAH BUKHARI - 15020" refreshedDate="46235.71296203704" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="20" xr:uid="{CA5F6DE5-CEA2-4E45-B954-94BF3111559B}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="K2:L22" sheet="Sheet5"/>
+    <worksheetSource ref="K2:L22" sheet="raw values"/>
   </cacheSource>
   <cacheFields count="2">
     <cacheField name="Prob" numFmtId="0">
@@ -4413,7 +4399,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="SYED UZAIR SHAH BUKHARI - 15020" refreshedDate="46235.713274652779" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="84" xr:uid="{A13CE6C0-AE51-544C-AEBA-6B56953E6821}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="O2:P86" sheet="Sheet5"/>
+    <worksheetSource ref="O2:P86" sheet="raw values"/>
   </cacheSource>
   <cacheFields count="2">
     <cacheField name="Prob" numFmtId="0">
@@ -4439,13 +4425,13 @@
 <file path=xl/pivotCache/pivotCacheDefinition6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="SYED UZAIR SHAH BUKHARI - 15020" refreshedDate="46235.724416435187" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="4" xr:uid="{85979681-CD81-7D49-8B4B-F3FFD2594E35}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="D1:H5" sheet="Sheet6"/>
+    <worksheetSource ref="D1:H5" sheet="summarized values"/>
   </cacheSource>
   <cacheFields count="5">
     <cacheField name="Simultaneous Arrival" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="3"/>
     </cacheField>
-    <cacheField name="Experiment 1" numFmtId="170">
+    <cacheField name="Experiment 1" numFmtId="164">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="6.1009916666666997E-2" maxValue="0.39399221666666701" count="4">
         <n v="0.28722328333333397"/>
         <n v="0.39399221666666701"/>
@@ -4453,7 +4439,7 @@
         <n v="6.1009916666666997E-2"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Experiment 2" numFmtId="170">
+    <cacheField name="Experiment 2" numFmtId="164">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="7.0382566666667007E-2" maxValue="0.39015898333333399" count="4">
         <n v="0.31595474999999995"/>
         <n v="0.39015898333333399"/>
@@ -4461,10 +4447,10 @@
         <n v="7.0382566666667007E-2"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Experiment 3" numFmtId="170">
+    <cacheField name="Experiment 3" numFmtId="164">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="8.0789583333332998E-2" maxValue="0.36107088333333398"/>
     </cacheField>
-    <cacheField name="Experiment 4" numFmtId="170">
+    <cacheField name="Experiment 4" numFmtId="164">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="2.5078765873015999E-2" maxValue="0.43577861111111299"/>
     </cacheField>
   </cacheFields>
@@ -5447,7 +5433,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5119AA26-79B5-6547-B249-38A3177BC80D}" name="PivotTable1" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5119AA26-79B5-6547-B249-38A3177BC80D}" name="PivotTable1" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="O7:P12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField dataField="1" showAll="0"/>
@@ -5500,7 +5486,191 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5B1D6295-02D1-284C-BE47-F22BB7322EE1}" name="PivotTable5" cacheId="28" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4028B6A7-71A9-EE4E-A17C-9E4DCDAF5D91}" name="PivotTable6" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:F9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="5">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" numFmtId="164" showAll="0">
+      <items count="5">
+        <item x="3"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" numFmtId="164" showAll="0">
+      <items count="5">
+        <item x="3"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="2"/>
+  </colFields>
+  <colItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{035FCF17-9505-D04F-86AE-47E07925DD26}" name="PivotTable3" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="F27:G32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="2">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Prob" fld="0" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DDD480FB-5004-1F4B-B51D-F83673BED8CE}" name="PivotTable2" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A27:B32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="2">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Prob" fld="0" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5B1D6295-02D1-284C-BE47-F22BB7322EE1}" name="PivotTable5" cacheId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="R27:S32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField dataField="1" showAll="0"/>
@@ -5552,8 +5722,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E503D647-ECC2-114A-82A2-79255C7E5B8E}" name="PivotTable4" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E503D647-ECC2-114A-82A2-79255C7E5B8E}" name="PivotTable4" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="J27:K32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField dataField="1" showAll="0"/>
@@ -5593,190 +5763,6 @@
   <dataFields count="1">
     <dataField name="Sum of Prob" fld="0" baseField="0" baseItem="0"/>
   </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{035FCF17-9505-D04F-86AE-47E07925DD26}" name="PivotTable3" cacheId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="F27:G32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="2">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Prob" fld="0" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DDD480FB-5004-1F4B-B51D-F83673BED8CE}" name="PivotTable2" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A27:B32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="2">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Prob" fld="0" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4028B6A7-71A9-EE4E-A17C-9E4DCDAF5D91}" name="PivotTable6" cacheId="33" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:F9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="5">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" numFmtId="170" showAll="0">
-      <items count="5">
-        <item x="3"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" numFmtId="170" showAll="0">
-      <items count="5">
-        <item x="3"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="170" showAll="0"/>
-    <pivotField numFmtId="170" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="2"/>
-  </colFields>
-  <colItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -8578,7 +8564,7 @@
       <c r="O8" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="P8" s="8">
+      <c r="P8">
         <v>0.34041754365079496</v>
       </c>
     </row>
@@ -8596,7 +8582,7 @@
       <c r="O9" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="P9" s="8">
+      <c r="P9">
         <v>0.43577861111111299</v>
       </c>
     </row>
@@ -8614,7 +8600,7 @@
       <c r="O10" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="P10" s="8">
+      <c r="P10">
         <v>0.19872507936507999</v>
       </c>
     </row>
@@ -8632,7 +8618,7 @@
       <c r="O11" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="P11" s="8">
+      <c r="P11">
         <v>2.5078765873015999E-2</v>
       </c>
     </row>
@@ -8650,7 +8636,7 @@
       <c r="O12" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="P12" s="8">
+      <c r="P12">
         <v>1.000000000000004</v>
       </c>
     </row>
@@ -9548,6 +9534,72 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C1934FE-FE83-0048-B607-884A9945FDE5}">
+  <dimension ref="A3:F9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B3" s="6" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="8">
+        <v>7.0382566666667007E-2</v>
+      </c>
+      <c r="C4" s="8">
+        <v>0.22350369999999997</v>
+      </c>
+      <c r="D4" s="8">
+        <v>0.31595474999999995</v>
+      </c>
+      <c r="E4" s="8">
+        <v>0.39015898333333399</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="10">
+        <v>6.1009916666666997E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="10">
+        <v>0.25777458333333403</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="10">
+        <v>0.28722328333333397</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="10">
+        <v>0.39399221666666701</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="10" t="s">
+        <v>135</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3270FDD7-B347-FE4A-9217-F7FEB4F37B1F}">
   <dimension ref="A1:S86"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -10542,19 +10594,19 @@
       <c r="A28" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B28">
         <v>0.33871326666666701</v>
       </c>
       <c r="F28" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="G28" s="8">
+      <c r="G28">
         <v>0.31595474999999995</v>
       </c>
       <c r="J28" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="K28" s="8">
+      <c r="K28">
         <v>0.28722328333333397</v>
       </c>
       <c r="N28" t="s">
@@ -10570,7 +10622,7 @@
       <c r="R28" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="S28" s="8">
+      <c r="S28">
         <v>0.34041754365079496</v>
       </c>
     </row>
@@ -10578,19 +10630,19 @@
       <c r="A29" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29">
         <v>0.36107088333333398</v>
       </c>
       <c r="F29" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="G29" s="8">
+      <c r="G29">
         <v>0.39015898333333399</v>
       </c>
       <c r="J29" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="K29" s="8">
+      <c r="K29">
         <v>0.39399221666666701</v>
       </c>
       <c r="N29" t="s">
@@ -10606,7 +10658,7 @@
       <c r="R29" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="S29" s="8">
+      <c r="S29">
         <v>0.43577861111111299</v>
       </c>
     </row>
@@ -10614,19 +10666,19 @@
       <c r="A30" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="B30" s="8">
+      <c r="B30">
         <v>0.21942626666666601</v>
       </c>
       <c r="F30" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="G30" s="8">
+      <c r="G30">
         <v>0.22350369999999997</v>
       </c>
       <c r="J30" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="K30" s="8">
+      <c r="K30">
         <v>0.25777458333333403</v>
       </c>
       <c r="N30" t="s">
@@ -10642,7 +10694,7 @@
       <c r="R30" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="S30" s="8">
+      <c r="S30">
         <v>0.19872507936507999</v>
       </c>
     </row>
@@ -10650,19 +10702,19 @@
       <c r="A31" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B31">
         <v>8.0789583333332998E-2</v>
       </c>
       <c r="F31" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="G31" s="8">
+      <c r="G31">
         <v>7.0382566666667007E-2</v>
       </c>
       <c r="J31" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="K31" s="8">
+      <c r="K31">
         <v>6.1009916666666997E-2</v>
       </c>
       <c r="N31" t="s">
@@ -10678,7 +10730,7 @@
       <c r="R31" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="S31" s="8">
+      <c r="S31">
         <v>2.5078765873015999E-2</v>
       </c>
     </row>
@@ -10686,19 +10738,19 @@
       <c r="A32" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="B32" s="8">
+      <c r="B32">
         <v>1</v>
       </c>
       <c r="F32" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="G32" s="8">
+      <c r="G32">
         <v>1.0000000000000009</v>
       </c>
       <c r="J32" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="K32" s="8">
+      <c r="K32">
         <v>1.000000000000002</v>
       </c>
       <c r="N32" t="s">
@@ -10714,7 +10766,7 @@
       <c r="R32" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="S32" s="8">
+      <c r="S32">
         <v>1.000000000000004</v>
       </c>
     </row>
@@ -11364,72 +11416,6 @@
       <c r="P86" t="str">
         <f t="shared" si="4"/>
         <v>"2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C1934FE-FE83-0048-B607-884A9945FDE5}">
-  <dimension ref="A3:F9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B3" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="B4" s="9">
-        <v>7.0382566666667007E-2</v>
-      </c>
-      <c r="C4" s="9">
-        <v>0.22350369999999997</v>
-      </c>
-      <c r="D4" s="9">
-        <v>0.31595474999999995</v>
-      </c>
-      <c r="E4" s="9">
-        <v>0.39015898333333399</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="11">
-        <v>6.1009916666666997E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="11">
-        <v>0.25777458333333403</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="11">
-        <v>0.28722328333333397</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="11">
-        <v>0.39399221666666701</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" s="11" t="s">
-        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -11467,16 +11453,16 @@
       <c r="D2">
         <v>0</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="8">
         <v>0.28722328333333397</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="8">
         <v>0.31595474999999995</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="8">
         <v>0.33871326666666701</v>
       </c>
-      <c r="H2" s="9">
+      <c r="H2" s="8">
         <v>0.34041754365079496</v>
       </c>
     </row>
@@ -11484,16 +11470,16 @@
       <c r="D3">
         <v>1</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="8">
         <v>0.39399221666666701</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="8">
         <v>0.39015898333333399</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="8">
         <v>0.36107088333333398</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="8">
         <v>0.43577861111111299</v>
       </c>
     </row>
@@ -11501,16 +11487,16 @@
       <c r="D4">
         <v>2</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="8">
         <v>0.25777458333333403</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4" s="8">
         <v>0.22350369999999997</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="8">
         <v>0.21942626666666601</v>
       </c>
-      <c r="H4" s="9">
+      <c r="H4" s="8">
         <v>0.19872507936507999</v>
       </c>
     </row>
@@ -11518,21 +11504,21 @@
       <c r="D5">
         <v>3</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="8">
         <v>6.1009916666666997E-2</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="8">
         <v>7.0382566666667007E-2</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="8">
         <v>8.0789583333332998E-2</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="8">
         <v>2.5078765873015999E-2</v>
       </c>
     </row>
     <row r="9" spans="4:8" ht="19" x14ac:dyDescent="0.2">
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="9" t="s">
         <v>138</v>
       </c>
     </row>

</xml_diff>